<commit_message>
EDU-45: class_manager: latest progress
</commit_message>
<xml_diff>
--- a/assets/deen/madrasa/class_manager.xlsx
+++ b/assets/deen/madrasa/class_manager.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SehhaDeveloper\src\l3\edu-journey\assets\deen\madrasa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C914B8B7-61D3-42EB-9119-954081B3D209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E012FC02-AC12-4D66-8F33-239C367575B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="10" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="205">
   <si>
     <t>Madrasa Class Dashboard</t>
   </si>
@@ -664,7 +664,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd\ mmm\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -926,13 +926,13 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -971,13 +971,13 @@
     <xf numFmtId="9" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1070,13 +1070,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF7EBC3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
@@ -1085,6 +1078,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF7EBC3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="H5" s="52">
         <f>COUNTIF(AttendanceTable[Student],$B$4)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" s="52">
         <f>COUNTIF(ProgressTable[Student],$B$4)</f>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="E20" s="3">
         <f>COUNTIFS(AttendanceTable[Student],$B$4,AttendanceTable[Status],D20)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -10837,12 +10837,22 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" ht="25" customHeight="1">
-      <c r="A8" s="29"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18"/>
+    <row r="8" spans="1:26">
+      <c r="A8" s="29">
+        <v>46277</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="18">
+        <v>0.47986111111111113</v>
+      </c>
       <c r="F8" s="17"/>
       <c r="G8" s="17"/>
       <c r="H8" s="19"/>
@@ -10865,12 +10875,22 @@
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
     </row>
-    <row r="9" spans="1:26" ht="25" customHeight="1">
-      <c r="A9" s="28"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="26"/>
+    <row r="9" spans="1:26">
+      <c r="A9" s="29">
+        <v>46277</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="26">
+        <v>0.47986111111111113</v>
+      </c>
       <c r="F9" s="25"/>
       <c r="G9" s="25"/>
       <c r="H9" s="27"/>
@@ -10893,12 +10913,22 @@
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" ht="25" customHeight="1">
-      <c r="A10" s="29"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="18"/>
+    <row r="10" spans="1:26">
+      <c r="A10" s="29">
+        <v>46277</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="18">
+        <v>0.47986111111111113</v>
+      </c>
       <c r="F10" s="17"/>
       <c r="G10" s="17"/>
       <c r="H10" s="19"/>
@@ -25712,13 +25742,13 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:I104">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>I5="Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>I5="Partly"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>I5="No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25805,7 +25835,7 @@
       <c r="H3" s="3"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:26" ht="14.1">
+    <row r="4" spans="1:26" ht="28.2">
       <c r="A4" s="23" t="s">
         <v>26</v>
       </c>
@@ -32807,10 +32837,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G204">
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>G5="Strong"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>G5="Needs Revision"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -40299,13 +40329,13 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F104">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>F5="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>F5="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>F5="Needs Revision"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>